<commit_message>
Auto commit - 08120934
</commit_message>
<xml_diff>
--- a/IM/202608_Service_Count_Report.xlsx
+++ b/IM/202608_Service_Count_Report.xlsx
@@ -2901,7 +2901,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="7">
-        <v>2026081255</v>
+        <v>2026081256</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -2940,7 +2940,7 @@
         <v>88</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="P11" s="7"/>
       <c r="Q11" s="7">
@@ -2949,9 +2949,7 @@
       <c r="R11" s="7">
         <v>747</v>
       </c>
-      <c r="S11" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S11" s="7"/>
       <c r="T11" s="7"/>
       <c r="U11" s="7"/>
       <c r="V11" s="7"/>
@@ -2973,7 +2971,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>2026081256</v>
+        <v>2026081255</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
@@ -3012,7 +3010,7 @@
         <v>88</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="P12" s="3"/>
       <c r="Q12" s="3">
@@ -3021,7 +3019,9 @@
       <c r="R12" s="3">
         <v>747</v>
       </c>
-      <c r="S12" s="3"/>
+      <c r="S12" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
@@ -3041,7 +3041,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="7">
-        <v>2026080104</v>
+        <v>2026080103</v>
       </c>
       <c r="C13" s="7">
         <v>1</v>
@@ -3080,7 +3080,7 @@
         <v>93</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="P13" s="7"/>
       <c r="Q13" s="7">
@@ -3089,7 +3089,9 @@
       <c r="R13" s="7">
         <v>2644</v>
       </c>
-      <c r="S13" s="7"/>
+      <c r="S13" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T13" s="7"/>
       <c r="U13" s="7"/>
       <c r="V13" s="7"/>
@@ -3111,7 +3113,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>2026080103</v>
+        <v>2026080104</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -3150,7 +3152,7 @@
         <v>93</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="P14" s="3"/>
       <c r="Q14" s="3">
@@ -3159,9 +3161,7 @@
       <c r="R14" s="3">
         <v>2644</v>
       </c>
-      <c r="S14" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
@@ -6223,7 +6223,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="3">
-        <v>2026080937</v>
+        <v>2026080936</v>
       </c>
       <c r="C60" s="3">
         <v>1</v>
@@ -6262,7 +6262,7 @@
         <v>253</v>
       </c>
       <c r="O60" s="3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="P60" s="3">
         <v>8160</v>
@@ -6273,7 +6273,9 @@
       <c r="R60" s="3">
         <v>26200</v>
       </c>
-      <c r="S60" s="3"/>
+      <c r="S60" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T60" s="3"/>
       <c r="U60" s="3"/>
       <c r="V60" s="3"/>
@@ -6295,7 +6297,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="7">
-        <v>2026080936</v>
+        <v>2026080937</v>
       </c>
       <c r="C61" s="7">
         <v>1</v>
@@ -6334,7 +6336,7 @@
         <v>253</v>
       </c>
       <c r="O61" s="7" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="P61" s="7">
         <v>8160</v>
@@ -6345,9 +6347,7 @@
       <c r="R61" s="7">
         <v>26200</v>
       </c>
-      <c r="S61" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S61" s="7"/>
       <c r="T61" s="7"/>
       <c r="U61" s="7"/>
       <c r="V61" s="7"/>
@@ -8059,7 +8059,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="7">
-        <v>2026080112</v>
+        <v>2026080113</v>
       </c>
       <c r="C87" s="7">
         <v>1</v>
@@ -8098,20 +8098,16 @@
         <v>321</v>
       </c>
       <c r="O87" s="7" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="P87" s="7"/>
       <c r="Q87" s="7"/>
       <c r="R87" s="7">
         <v>251357</v>
       </c>
-      <c r="S87" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S87" s="7"/>
       <c r="T87" s="7"/>
-      <c r="U87" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="U87" s="7"/>
       <c r="V87" s="7"/>
       <c r="W87" s="7"/>
       <c r="X87" s="7"/>
@@ -8127,7 +8123,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="3">
-        <v>2026080113</v>
+        <v>2026080112</v>
       </c>
       <c r="C88" s="3">
         <v>1</v>
@@ -8166,16 +8162,20 @@
         <v>321</v>
       </c>
       <c r="O88" s="3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="P88" s="3"/>
       <c r="Q88" s="3"/>
       <c r="R88" s="3">
         <v>251357</v>
       </c>
-      <c r="S88" s="3"/>
+      <c r="S88" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T88" s="3"/>
-      <c r="U88" s="3"/>
+      <c r="U88" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="V88" s="3"/>
       <c r="W88" s="3"/>
       <c r="X88" s="3"/>
@@ -14371,7 +14371,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="3">
-        <v>2026081171</v>
+        <v>2026081285</v>
       </c>
       <c r="C180" s="3">
         <v>1</v>
@@ -14394,12 +14394,8 @@
       <c r="I180" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="J180" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="K180" s="3" t="s">
-        <v>191</v>
-      </c>
+      <c r="J180" s="3"/>
+      <c r="K180" s="3"/>
       <c r="L180" s="6" t="s">
         <v>183</v>
       </c>
@@ -14410,14 +14406,16 @@
         <v>575</v>
       </c>
       <c r="O180" s="3" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="P180" s="3"/>
       <c r="Q180" s="3"/>
       <c r="R180" s="3">
         <v>0</v>
       </c>
-      <c r="S180" s="3"/>
+      <c r="S180" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T180" s="3"/>
       <c r="U180" s="3"/>
       <c r="V180" s="3"/>
@@ -14425,7 +14423,7 @@
       <c r="X180" s="3"/>
       <c r="Y180" s="3"/>
       <c r="Z180" s="6" t="s">
-        <v>576</v>
+        <v>186</v>
       </c>
       <c r="AA180" s="3" t="s">
         <v>40</v>
@@ -14439,7 +14437,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="7">
-        <v>2026081285</v>
+        <v>2026081171</v>
       </c>
       <c r="C181" s="7">
         <v>1</v>
@@ -14462,8 +14460,12 @@
       <c r="I181" s="7" t="s">
         <v>573</v>
       </c>
-      <c r="J181" s="7"/>
-      <c r="K181" s="7"/>
+      <c r="J181" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="K181" s="7" t="s">
+        <v>191</v>
+      </c>
       <c r="L181" s="8" t="s">
         <v>183</v>
       </c>
@@ -14474,16 +14476,14 @@
         <v>575</v>
       </c>
       <c r="O181" s="7" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="P181" s="7"/>
       <c r="Q181" s="7"/>
       <c r="R181" s="7">
         <v>0</v>
       </c>
-      <c r="S181" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S181" s="7"/>
       <c r="T181" s="7"/>
       <c r="U181" s="7"/>
       <c r="V181" s="7"/>
@@ -14491,7 +14491,7 @@
       <c r="X181" s="7"/>
       <c r="Y181" s="7"/>
       <c r="Z181" s="8" t="s">
-        <v>186</v>
+        <v>576</v>
       </c>
       <c r="AA181" s="7" t="s">
         <v>40</v>

</xml_diff>